<commit_message>
Added Weekly Scope ticket
</commit_message>
<xml_diff>
--- a/Weekly_Scope_Project_Development_Plan.xlsx
+++ b/Weekly_Scope_Project_Development_Plan.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anjani\TaxConsultionOfficeManagement\TaxConsultingOfficeManagmement\ISoftTechSolutions\TaxConsultencyOfficeManagement\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2BCAC3-EAF7-4BD1-873A-CCA0A1AFFC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Objectives" sheetId="1" r:id="rId1"/>
@@ -15,12 +21,12 @@
     <sheet name="Issues" sheetId="6" r:id="rId6"/>
     <sheet name="Meetings" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="94">
   <si>
     <t>High-Level Goals</t>
   </si>
@@ -130,15 +136,6 @@
     <t>Milestone 3</t>
   </si>
   <si>
-    <t>Description of milestone 1</t>
-  </si>
-  <si>
-    <t>Description of milestone 2</t>
-  </si>
-  <si>
-    <t>Description of milestone 3</t>
-  </si>
-  <si>
     <t>[Due Date]</t>
   </si>
   <si>
@@ -284,13 +281,40 @@
   </si>
   <si>
     <t>[Outcome]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer detail add with Validation </t>
+  </si>
+  <si>
+    <t>Add Orgnization with Employee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not Started </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Save Detail of Tax  Filling </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not Sarted </t>
+  </si>
+  <si>
+    <t>Milestone 4</t>
+  </si>
+  <si>
+    <t>Deploy on Cloud with Tax Service</t>
+  </si>
+  <si>
+    <t>K8S cluster setup with Depoy all Service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,24 +366,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -397,7 +431,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -431,6 +465,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -465,9 +500,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -640,26 +676,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -670,11 +706,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="29.453125" customWidth="1"/>
+    <col min="2" max="2" width="33.6328125" customWidth="1"/>
+    <col min="3" max="3" width="31.1796875" customWidth="1"/>
+    <col min="4" max="4" width="27.6328125" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="24.54296875" customWidth="1"/>
+    <col min="7" max="7" width="16.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -697,7 +742,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -720,7 +765,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -743,7 +788,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -766,7 +811,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -795,11 +840,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28.81640625" customWidth="1"/>
+    <col min="2" max="2" width="36.36328125" customWidth="1"/>
+    <col min="3" max="3" width="30.36328125" customWidth="1"/>
+    <col min="4" max="4" width="35.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
@@ -813,46 +864,74 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
+        <v>85</v>
+      </c>
+      <c r="C2" s="2">
+        <v>45480</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
+        <v>86</v>
+      </c>
+      <c r="C3" s="2">
+        <v>45487</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" t="s">
-        <v>39</v>
+        <v>88</v>
+      </c>
+      <c r="C4" s="2">
+        <v>45500</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="2">
+        <v>45487</v>
+      </c>
+      <c r="D5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="3">
+        <v>45500</v>
+      </c>
+      <c r="D6" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -861,13 +940,13 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
@@ -879,43 +958,43 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
         <v>43</v>
       </c>
-      <c r="B4" t="s">
-        <v>46</v>
-      </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>
@@ -927,64 +1006,69 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" customWidth="1"/>
+    <col min="2" max="2" width="32.1796875" customWidth="1"/>
+    <col min="3" max="3" width="38.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>52</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>55</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -993,76 +1077,76 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
         <v>64</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>67</v>
       </c>
-      <c r="C2" t="s">
-        <v>70</v>
-      </c>
       <c r="D2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
         <v>65</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>68</v>
       </c>
-      <c r="C3" t="s">
-        <v>71</v>
-      </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
         <v>66</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>69</v>
       </c>
-      <c r="C4" t="s">
-        <v>72</v>
-      </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1071,76 +1155,76 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>75</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>76</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
         <v>81</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" t="s">
         <v>84</v>
-      </c>
-      <c r="D2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>